<commit_message>
feat: cache-bust + relacionados, skeleton, selo %, ordenar/filtrar, obs/limpar carrinho
- Cache-busting (?v=) em CSS/JS no index e nas páginas de categoria — corrige usuário vendo versão antiga
- Selo de % de desconto no card (vermelho) além da tag/preço
- Pop-up: produtos relacionados (mesma categoria) + skeleton (ícone da logo) enquanto a imagem carrega
- Skeleton também nos cards (isotipo + shimmer atrás das fotos)
- Página de categoria: filtro por tag (Todos/Em estoque/Promoção) + ordenar (preço/nome)
- Carrinho: campo de observação (entra na mensagem do WhatsApp) + botão Limpar carrinho (com confirmação)
- Gerador: TAG 'oferta' tratada como promoção; dados reais do Excel (TAG/PRECO_PROMO)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Catalogo_Produtos.xlsx
+++ b/Catalogo_Produtos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Felipe.bortolini\Documents\Caieiras Pesca\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B888679-EC98-4523-B78F-96E9030C20CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{143BCE2A-A77B-4124-92AC-E42B50813D6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1311EB0D-21A8-4CC1-B824-0871D74D03FF}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="34">
   <si>
     <t>CATEGORA</t>
   </si>
@@ -112,6 +112,21 @@
   </si>
   <si>
     <t>C:\Users\Felipe.bortolini\Documents\Caieiras Pesca\imagens\VARAS\ALBATROZ_VIPER</t>
+  </si>
+  <si>
+    <t>PRECO_PROMO</t>
+  </si>
+  <si>
+    <t>TAG</t>
+  </si>
+  <si>
+    <t>Promoção</t>
+  </si>
+  <si>
+    <t>Em estoque</t>
+  </si>
+  <si>
+    <t>Indisponivel</t>
   </si>
 </sst>
 </file>
@@ -121,8 +136,16 @@
   <numFmts count="1">
     <numFmt numFmtId="8" formatCode="&quot;R$&quot;\ #,##0.00;[Red]\-&quot;R$&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -150,9 +173,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -171,14 +195,16 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{73CAE26C-5F31-48AB-B16F-0D4A0A3558CF}" name="Tabela1" displayName="Tabela1" ref="A1:E8" totalsRowShown="0">
-  <autoFilter ref="A1:E8" xr:uid="{73CAE26C-5F31-48AB-B16F-0D4A0A3558CF}"/>
-  <tableColumns count="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{73CAE26C-5F31-48AB-B16F-0D4A0A3558CF}" name="Tabela1" displayName="Tabela1" ref="A1:G8" totalsRowShown="0">
+  <autoFilter ref="A1:G8" xr:uid="{73CAE26C-5F31-48AB-B16F-0D4A0A3558CF}"/>
+  <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{B47AC1F9-FE40-474D-8763-162FF4DDD9CF}" name="CATEGORA"/>
     <tableColumn id="2" xr3:uid="{EAFE3CB5-8C53-4A31-8CDF-4059EF76B468}" name="PRODUTO"/>
     <tableColumn id="3" xr3:uid="{EA923502-C285-43D2-AD50-0CE5A0B63C9C}" name="DESCRIÇÃO"/>
     <tableColumn id="4" xr3:uid="{A6F22F24-4811-494C-9426-76AD1CB116F6}" name="VALOR"/>
     <tableColumn id="5" xr3:uid="{5A327B39-121D-4882-B7D3-FFEC5A5378EB}" name="PASTA_IMAGENS"/>
+    <tableColumn id="6" xr3:uid="{5EB18D88-9A08-449A-960A-2380B6389969}" name="TAG"/>
+    <tableColumn id="7" xr3:uid="{F0DA816A-6023-4630-8B09-C45B8776C57B}" name="PRECO_PROMO"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight13" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -481,7 +507,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CEE83D0-8926-48A7-A1AD-CAFC3803DB9C}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
@@ -489,9 +515,10 @@
     <col min="3" max="3" width="31.42578125" customWidth="1"/>
     <col min="4" max="4" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="119.42578125" customWidth="1"/>
+    <col min="6" max="6" width="15.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -507,8 +534,14 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F1" t="s">
+        <v>30</v>
+      </c>
+      <c r="G1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -524,8 +557,14 @@
       <c r="E2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F2" t="s">
+        <v>31</v>
+      </c>
+      <c r="G2" s="1">
+        <v>39.9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -541,8 +580,11 @@
       <c r="E3" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -558,8 +600,11 @@
       <c r="E4" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -575,8 +620,11 @@
       <c r="E5" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -592,8 +640,11 @@
       <c r="E6" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -609,8 +660,11 @@
       <c r="E7" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -626,6 +680,12 @@
       <c r="E8" t="s">
         <v>28</v>
       </c>
+      <c r="F8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E13" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>